<commit_message>
update excel for foods
</commit_message>
<xml_diff>
--- a/cache/sepidar_food_code.xlsx
+++ b/cache/sepidar_food_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dorsa-Co\Desktop\temp\seketala\cache\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA2439C-E691-4D0C-ABC7-FE05FEBB1B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26D4D3D6-1B0E-4CA4-AF82-6262BA7B5F59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1380" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="568">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="624">
   <si>
     <t>كد</t>
   </si>
@@ -1729,6 +1729,174 @@
   </si>
   <si>
     <t>سالاد کلم</t>
+  </si>
+  <si>
+    <t>1100065</t>
+  </si>
+  <si>
+    <t>1100066</t>
+  </si>
+  <si>
+    <t>آب معدني 300 سي سي</t>
+  </si>
+  <si>
+    <t>1100067</t>
+  </si>
+  <si>
+    <t>خانواده كوكا با ليوان</t>
+  </si>
+  <si>
+    <t>1100068</t>
+  </si>
+  <si>
+    <t>خانواده فانتا با ليوان</t>
+  </si>
+  <si>
+    <t>1100069</t>
+  </si>
+  <si>
+    <t>خانواده اسپرايت با ليوان</t>
+  </si>
+  <si>
+    <t>1100070</t>
+  </si>
+  <si>
+    <t>خانواده ليموناد فانتا با ليوان</t>
+  </si>
+  <si>
+    <t>1100071</t>
+  </si>
+  <si>
+    <t>خانواده مشكي زيرو با ليوان</t>
+  </si>
+  <si>
+    <t>1100072</t>
+  </si>
+  <si>
+    <t>خانواده شاه توت با ليوان</t>
+  </si>
+  <si>
+    <t>1100073</t>
+  </si>
+  <si>
+    <t>قوطي كوكا با ليوان</t>
+  </si>
+  <si>
+    <t>1100074</t>
+  </si>
+  <si>
+    <t>قوطي فانتا با ليوان</t>
+  </si>
+  <si>
+    <t>1100075</t>
+  </si>
+  <si>
+    <t>قوطي زيرو با ليوان</t>
+  </si>
+  <si>
+    <t>1100076</t>
+  </si>
+  <si>
+    <t>قوطي ليموناد خوشگوار با ليوان</t>
+  </si>
+  <si>
+    <t>1100077</t>
+  </si>
+  <si>
+    <t>قوطي اسپرايت با ليوان</t>
+  </si>
+  <si>
+    <t>1100078</t>
+  </si>
+  <si>
+    <t>هي دي ليمو با ليوان</t>
+  </si>
+  <si>
+    <t>1100079</t>
+  </si>
+  <si>
+    <t xml:space="preserve">هي دي هلو با ليوان </t>
+  </si>
+  <si>
+    <t>1100080</t>
+  </si>
+  <si>
+    <t>هي دي استوايي با ليوان</t>
+  </si>
+  <si>
+    <t>1100081</t>
+  </si>
+  <si>
+    <t>هي دي كلاسيك با ليوان</t>
+  </si>
+  <si>
+    <t>1100082</t>
+  </si>
+  <si>
+    <t>هافنبرگ كاكتوس با ليوان</t>
+  </si>
+  <si>
+    <t>1100083</t>
+  </si>
+  <si>
+    <t>دوغ خوشگوار با ليوان</t>
+  </si>
+  <si>
+    <t>هي دي كلاسيك</t>
+  </si>
+  <si>
+    <t>1100056</t>
+  </si>
+  <si>
+    <t>كالاي تست ارزش افزوده</t>
+  </si>
+  <si>
+    <t>1100057</t>
+  </si>
+  <si>
+    <t>بوفالو وينگز فروش</t>
+  </si>
+  <si>
+    <t>1100058</t>
+  </si>
+  <si>
+    <t>سالاد سزار مرغ فروش</t>
+  </si>
+  <si>
+    <t>1100059</t>
+  </si>
+  <si>
+    <t>خوراك فيله سوخاري دو تكه</t>
+  </si>
+  <si>
+    <t>1100060</t>
+  </si>
+  <si>
+    <t>سالاد كلم تكي</t>
+  </si>
+  <si>
+    <t>1100061</t>
+  </si>
+  <si>
+    <t>سس خردل تكي</t>
+  </si>
+  <si>
+    <t>1100062</t>
+  </si>
+  <si>
+    <t>سس فرانسوي تكي</t>
+  </si>
+  <si>
+    <t>1100063</t>
+  </si>
+  <si>
+    <t>خانواده ليمويي</t>
+  </si>
+  <si>
+    <t>1100064</t>
+  </si>
+  <si>
+    <t>خانواده شاتوت</t>
   </si>
 </sst>
 </file>
@@ -1754,7 +1922,7 @@
       <name val="Tahoma"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1764,6 +1932,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFECF4FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7F1FF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1780,11 +1954,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="4" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2065,7 +2242,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B288"/>
+  <dimension ref="A1:R332"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" customWidth="1"/>
@@ -4376,6 +4553,964 @@
         <v>567</v>
       </c>
     </row>
+    <row r="289" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A289" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B289" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="C289" s="2"/>
+      <c r="F289" s="2"/>
+      <c r="G289" s="2"/>
+      <c r="H289" s="2"/>
+      <c r="I289" s="2"/>
+      <c r="J289" s="2"/>
+      <c r="K289" s="2"/>
+      <c r="L289" s="5"/>
+      <c r="M289" s="2"/>
+      <c r="N289" s="5"/>
+      <c r="O289" s="2"/>
+      <c r="P289" s="2"/>
+      <c r="Q289" s="2"/>
+      <c r="R289" s="2"/>
+    </row>
+    <row r="290" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A290" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B290" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C290" s="3"/>
+      <c r="F290" s="3"/>
+      <c r="G290" s="3"/>
+      <c r="H290" s="3"/>
+      <c r="I290" s="3"/>
+      <c r="J290" s="3"/>
+      <c r="K290" s="3"/>
+      <c r="L290" s="6"/>
+      <c r="M290" s="3"/>
+      <c r="N290" s="6"/>
+      <c r="O290" s="3"/>
+      <c r="P290" s="3"/>
+      <c r="Q290" s="3"/>
+      <c r="R290" s="3"/>
+    </row>
+    <row r="291" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A291" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B291" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="C291" s="3"/>
+      <c r="F291" s="3"/>
+      <c r="G291" s="3"/>
+      <c r="H291" s="3"/>
+      <c r="I291" s="3"/>
+      <c r="J291" s="3"/>
+      <c r="K291" s="3"/>
+      <c r="L291" s="6"/>
+      <c r="M291" s="3"/>
+      <c r="N291" s="6"/>
+      <c r="O291" s="3"/>
+      <c r="P291" s="3"/>
+      <c r="Q291" s="3"/>
+      <c r="R291" s="3"/>
+    </row>
+    <row r="292" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A292" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B292" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="C292" s="2"/>
+      <c r="F292" s="2"/>
+      <c r="G292" s="2"/>
+      <c r="H292" s="2"/>
+      <c r="I292" s="2"/>
+      <c r="J292" s="2"/>
+      <c r="K292" s="2"/>
+      <c r="L292" s="5"/>
+      <c r="M292" s="2"/>
+      <c r="N292" s="5"/>
+      <c r="O292" s="2"/>
+      <c r="P292" s="2"/>
+      <c r="Q292" s="2"/>
+      <c r="R292" s="2"/>
+    </row>
+    <row r="293" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A293" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B293" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="C293" s="3"/>
+      <c r="F293" s="3"/>
+      <c r="G293" s="3"/>
+      <c r="H293" s="3"/>
+      <c r="I293" s="3"/>
+      <c r="J293" s="3"/>
+      <c r="K293" s="3"/>
+      <c r="L293" s="6"/>
+      <c r="M293" s="3"/>
+      <c r="N293" s="6"/>
+      <c r="O293" s="3"/>
+      <c r="P293" s="3"/>
+      <c r="Q293" s="3"/>
+      <c r="R293" s="3"/>
+    </row>
+    <row r="294" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A294" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B294" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="C294" s="2"/>
+      <c r="F294" s="2"/>
+      <c r="G294" s="2"/>
+      <c r="H294" s="2"/>
+      <c r="I294" s="2"/>
+      <c r="J294" s="2"/>
+      <c r="K294" s="2"/>
+      <c r="L294" s="5"/>
+      <c r="M294" s="2"/>
+      <c r="N294" s="5"/>
+      <c r="O294" s="2"/>
+      <c r="P294" s="2"/>
+      <c r="Q294" s="2"/>
+      <c r="R294" s="2"/>
+    </row>
+    <row r="295" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A295" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B295" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="C295" s="3"/>
+      <c r="F295" s="3"/>
+      <c r="G295" s="3"/>
+      <c r="H295" s="3"/>
+      <c r="I295" s="3"/>
+      <c r="J295" s="3"/>
+      <c r="K295" s="3"/>
+      <c r="L295" s="6"/>
+      <c r="M295" s="3"/>
+      <c r="N295" s="6"/>
+      <c r="O295" s="3"/>
+      <c r="P295" s="3"/>
+      <c r="Q295" s="3"/>
+      <c r="R295" s="3"/>
+    </row>
+    <row r="296" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A296" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B296" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="C296" s="2"/>
+      <c r="F296" s="2"/>
+      <c r="G296" s="2"/>
+      <c r="H296" s="2"/>
+      <c r="I296" s="2"/>
+      <c r="J296" s="2"/>
+      <c r="K296" s="2"/>
+      <c r="L296" s="5"/>
+      <c r="M296" s="2"/>
+      <c r="N296" s="5"/>
+      <c r="O296" s="2"/>
+      <c r="P296" s="2"/>
+      <c r="Q296" s="2"/>
+      <c r="R296" s="2"/>
+    </row>
+    <row r="297" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A297" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B297" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C297" s="3"/>
+      <c r="F297" s="3"/>
+      <c r="G297" s="3"/>
+      <c r="H297" s="3"/>
+      <c r="I297" s="3"/>
+      <c r="J297" s="3"/>
+      <c r="K297" s="3"/>
+      <c r="L297" s="6"/>
+      <c r="M297" s="3"/>
+      <c r="N297" s="6"/>
+      <c r="O297" s="3"/>
+      <c r="P297" s="3"/>
+      <c r="Q297" s="3"/>
+      <c r="R297" s="3"/>
+    </row>
+    <row r="298" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A298" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B298" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C298" s="2"/>
+      <c r="F298" s="2"/>
+      <c r="G298" s="2"/>
+      <c r="H298" s="2"/>
+      <c r="I298" s="2"/>
+      <c r="J298" s="2"/>
+      <c r="K298" s="2"/>
+      <c r="L298" s="5"/>
+      <c r="M298" s="2"/>
+      <c r="N298" s="5"/>
+      <c r="O298" s="2"/>
+      <c r="P298" s="2"/>
+      <c r="Q298" s="2"/>
+      <c r="R298" s="2"/>
+    </row>
+    <row r="299" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A299" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B299" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="C299" s="3"/>
+      <c r="F299" s="3"/>
+      <c r="G299" s="3"/>
+      <c r="H299" s="3"/>
+      <c r="I299" s="3"/>
+      <c r="J299" s="3"/>
+      <c r="K299" s="3"/>
+      <c r="L299" s="6"/>
+      <c r="M299" s="3"/>
+      <c r="N299" s="6"/>
+      <c r="O299" s="3"/>
+      <c r="P299" s="3"/>
+      <c r="Q299" s="3"/>
+      <c r="R299" s="3"/>
+    </row>
+    <row r="300" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A300" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B300" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="C300" s="2"/>
+      <c r="F300" s="2"/>
+      <c r="G300" s="2"/>
+      <c r="H300" s="2"/>
+      <c r="I300" s="2"/>
+      <c r="J300" s="2"/>
+      <c r="K300" s="2"/>
+      <c r="L300" s="5"/>
+      <c r="M300" s="2"/>
+      <c r="N300" s="5"/>
+      <c r="O300" s="2"/>
+      <c r="P300" s="2"/>
+      <c r="Q300" s="2"/>
+      <c r="R300" s="2"/>
+    </row>
+    <row r="301" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A301" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B301" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C301" s="3"/>
+      <c r="F301" s="3"/>
+      <c r="G301" s="3"/>
+      <c r="H301" s="3"/>
+      <c r="I301" s="3"/>
+      <c r="J301" s="3"/>
+      <c r="K301" s="3"/>
+      <c r="L301" s="6"/>
+      <c r="M301" s="3"/>
+      <c r="N301" s="6"/>
+      <c r="O301" s="3"/>
+      <c r="P301" s="3"/>
+      <c r="Q301" s="3"/>
+      <c r="R301" s="3"/>
+    </row>
+    <row r="302" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A302" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B302" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="C302" s="2"/>
+      <c r="F302" s="2"/>
+      <c r="G302" s="2"/>
+      <c r="H302" s="2"/>
+      <c r="I302" s="2"/>
+      <c r="J302" s="2"/>
+      <c r="K302" s="2"/>
+      <c r="L302" s="5"/>
+      <c r="M302" s="2"/>
+      <c r="N302" s="5"/>
+      <c r="O302" s="2"/>
+      <c r="P302" s="2"/>
+      <c r="Q302" s="2"/>
+      <c r="R302" s="2"/>
+    </row>
+    <row r="303" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A303" s="3" t="s">
+        <v>606</v>
+      </c>
+      <c r="B303" s="3" t="s">
+        <v>607</v>
+      </c>
+      <c r="C303" s="3"/>
+      <c r="F303" s="3"/>
+      <c r="G303" s="3"/>
+      <c r="H303" s="3"/>
+      <c r="I303" s="3"/>
+      <c r="J303" s="3"/>
+      <c r="K303" s="3"/>
+      <c r="L303" s="6"/>
+      <c r="M303" s="3"/>
+      <c r="N303" s="6"/>
+      <c r="O303" s="3"/>
+      <c r="P303" s="3"/>
+      <c r="Q303" s="3"/>
+      <c r="R303" s="3"/>
+    </row>
+    <row r="304" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A304" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="B304" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="C304" s="2"/>
+      <c r="F304" s="2"/>
+      <c r="G304" s="2"/>
+      <c r="H304" s="2"/>
+      <c r="I304" s="2"/>
+      <c r="J304" s="2"/>
+      <c r="K304" s="2"/>
+      <c r="L304" s="5"/>
+      <c r="M304" s="2"/>
+      <c r="N304" s="5"/>
+      <c r="O304" s="2"/>
+      <c r="P304" s="2"/>
+      <c r="Q304" s="2"/>
+      <c r="R304" s="2"/>
+    </row>
+    <row r="305" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A305" s="3" t="s">
+        <v>610</v>
+      </c>
+      <c r="B305" s="3" t="s">
+        <v>611</v>
+      </c>
+      <c r="C305" s="3"/>
+      <c r="F305" s="3"/>
+      <c r="G305" s="3"/>
+      <c r="H305" s="3"/>
+      <c r="I305" s="3"/>
+      <c r="J305" s="3"/>
+      <c r="K305" s="3"/>
+      <c r="L305" s="6"/>
+      <c r="M305" s="3"/>
+      <c r="N305" s="6"/>
+      <c r="O305" s="3"/>
+      <c r="P305" s="3"/>
+      <c r="Q305" s="3"/>
+      <c r="R305" s="3"/>
+    </row>
+    <row r="306" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A306" s="2" t="s">
+        <v>612</v>
+      </c>
+      <c r="B306" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="C306" s="2"/>
+      <c r="F306" s="2"/>
+      <c r="G306" s="2"/>
+      <c r="H306" s="2"/>
+      <c r="I306" s="2"/>
+      <c r="J306" s="2"/>
+      <c r="K306" s="2"/>
+      <c r="L306" s="5"/>
+      <c r="M306" s="2"/>
+      <c r="N306" s="5"/>
+      <c r="O306" s="2"/>
+      <c r="P306" s="2"/>
+      <c r="Q306" s="2"/>
+      <c r="R306" s="2"/>
+    </row>
+    <row r="307" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A307" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="B307" s="3" t="s">
+        <v>615</v>
+      </c>
+      <c r="C307" s="3"/>
+      <c r="F307" s="3"/>
+      <c r="G307" s="3"/>
+      <c r="H307" s="3"/>
+      <c r="I307" s="3"/>
+      <c r="J307" s="3"/>
+      <c r="K307" s="3"/>
+      <c r="L307" s="6"/>
+      <c r="M307" s="3"/>
+      <c r="N307" s="6"/>
+      <c r="O307" s="3"/>
+      <c r="P307" s="3"/>
+      <c r="Q307" s="3"/>
+      <c r="R307" s="3"/>
+    </row>
+    <row r="308" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A308" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="B308" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="C308" s="2"/>
+      <c r="F308" s="2"/>
+      <c r="G308" s="2"/>
+      <c r="H308" s="2"/>
+      <c r="I308" s="2"/>
+      <c r="J308" s="2"/>
+      <c r="K308" s="2"/>
+      <c r="L308" s="5"/>
+      <c r="M308" s="2"/>
+      <c r="N308" s="5"/>
+      <c r="O308" s="2"/>
+      <c r="P308" s="2"/>
+      <c r="Q308" s="2"/>
+      <c r="R308" s="2"/>
+    </row>
+    <row r="309" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A309" s="3" t="s">
+        <v>618</v>
+      </c>
+      <c r="B309" s="3" t="s">
+        <v>619</v>
+      </c>
+      <c r="C309" s="3"/>
+      <c r="F309" s="3"/>
+      <c r="G309" s="3"/>
+      <c r="H309" s="3"/>
+      <c r="I309" s="3"/>
+      <c r="J309" s="3"/>
+      <c r="K309" s="3"/>
+      <c r="L309" s="6"/>
+      <c r="M309" s="3"/>
+      <c r="N309" s="6"/>
+      <c r="O309" s="3"/>
+      <c r="P309" s="3"/>
+      <c r="Q309" s="3"/>
+      <c r="R309" s="3"/>
+    </row>
+    <row r="310" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A310" s="2" t="s">
+        <v>620</v>
+      </c>
+      <c r="B310" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="C310" s="2"/>
+      <c r="F310" s="2"/>
+      <c r="G310" s="2"/>
+      <c r="H310" s="2"/>
+      <c r="I310" s="2"/>
+      <c r="J310" s="2"/>
+      <c r="K310" s="2"/>
+      <c r="L310" s="5"/>
+      <c r="M310" s="2"/>
+      <c r="N310" s="5"/>
+      <c r="O310" s="2"/>
+      <c r="P310" s="2"/>
+      <c r="Q310" s="2"/>
+      <c r="R310" s="2"/>
+    </row>
+    <row r="311" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A311" s="3" t="s">
+        <v>622</v>
+      </c>
+      <c r="B311" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="C311" s="3"/>
+      <c r="F311" s="3"/>
+      <c r="G311" s="3"/>
+      <c r="H311" s="3"/>
+      <c r="I311" s="3"/>
+      <c r="J311" s="3"/>
+      <c r="K311" s="3"/>
+      <c r="L311" s="6"/>
+      <c r="M311" s="3"/>
+      <c r="N311" s="6"/>
+      <c r="O311" s="3"/>
+      <c r="P311" s="3"/>
+      <c r="Q311" s="3"/>
+      <c r="R311" s="3"/>
+    </row>
+    <row r="312" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A312" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="B312" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C312" s="2"/>
+      <c r="F312" s="2"/>
+      <c r="G312" s="2"/>
+      <c r="H312" s="2"/>
+      <c r="I312" s="2"/>
+      <c r="J312" s="2"/>
+      <c r="K312" s="2"/>
+      <c r="L312" s="5"/>
+      <c r="M312" s="2"/>
+      <c r="N312" s="5"/>
+      <c r="O312" s="2"/>
+      <c r="P312" s="2"/>
+      <c r="Q312" s="2"/>
+      <c r="R312" s="2"/>
+    </row>
+    <row r="313" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A313" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="B313" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C313" s="3"/>
+      <c r="F313" s="3"/>
+      <c r="G313" s="3"/>
+      <c r="H313" s="3"/>
+      <c r="I313" s="3"/>
+      <c r="J313" s="3"/>
+      <c r="K313" s="3"/>
+      <c r="L313" s="6"/>
+      <c r="M313" s="3"/>
+      <c r="N313" s="6"/>
+      <c r="O313" s="3"/>
+      <c r="P313" s="3"/>
+      <c r="Q313" s="3"/>
+      <c r="R313" s="3"/>
+    </row>
+    <row r="314" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A314" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="B314" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="C314" s="2"/>
+      <c r="F314" s="2"/>
+      <c r="G314" s="2"/>
+      <c r="H314" s="2"/>
+      <c r="I314" s="2"/>
+      <c r="J314" s="2"/>
+      <c r="K314" s="2"/>
+      <c r="L314" s="5"/>
+      <c r="M314" s="2"/>
+      <c r="N314" s="5"/>
+      <c r="O314" s="2"/>
+      <c r="P314" s="2"/>
+      <c r="Q314" s="2"/>
+      <c r="R314" s="2"/>
+    </row>
+    <row r="315" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A315" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="B315" s="3" t="s">
+        <v>574</v>
+      </c>
+      <c r="C315" s="3"/>
+      <c r="F315" s="3"/>
+      <c r="G315" s="3"/>
+      <c r="H315" s="3"/>
+      <c r="I315" s="3"/>
+      <c r="J315" s="3"/>
+      <c r="K315" s="3"/>
+      <c r="L315" s="6"/>
+      <c r="M315" s="3"/>
+      <c r="N315" s="6"/>
+      <c r="O315" s="3"/>
+      <c r="P315" s="3"/>
+      <c r="Q315" s="3"/>
+      <c r="R315" s="3"/>
+    </row>
+    <row r="316" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A316" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="B316" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="C316" s="2"/>
+      <c r="F316" s="2"/>
+      <c r="G316" s="2"/>
+      <c r="H316" s="2"/>
+      <c r="I316" s="2"/>
+      <c r="J316" s="2"/>
+      <c r="K316" s="2"/>
+      <c r="L316" s="5"/>
+      <c r="M316" s="2"/>
+      <c r="N316" s="5"/>
+      <c r="O316" s="2"/>
+      <c r="P316" s="2"/>
+      <c r="Q316" s="2"/>
+      <c r="R316" s="2"/>
+    </row>
+    <row r="317" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A317" s="3" t="s">
+        <v>577</v>
+      </c>
+      <c r="B317" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="C317" s="3"/>
+      <c r="F317" s="3"/>
+      <c r="G317" s="3"/>
+      <c r="H317" s="3"/>
+      <c r="I317" s="3"/>
+      <c r="J317" s="3"/>
+      <c r="K317" s="3"/>
+      <c r="L317" s="6"/>
+      <c r="M317" s="3"/>
+      <c r="N317" s="6"/>
+      <c r="O317" s="3"/>
+      <c r="P317" s="3"/>
+      <c r="Q317" s="3"/>
+      <c r="R317" s="3"/>
+    </row>
+    <row r="318" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A318" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="B318" s="2" t="s">
+        <v>580</v>
+      </c>
+      <c r="C318" s="2"/>
+      <c r="F318" s="2"/>
+      <c r="G318" s="2"/>
+      <c r="H318" s="2"/>
+      <c r="I318" s="2"/>
+      <c r="J318" s="2"/>
+      <c r="K318" s="2"/>
+      <c r="L318" s="5"/>
+      <c r="M318" s="2"/>
+      <c r="N318" s="5"/>
+      <c r="O318" s="2"/>
+      <c r="P318" s="2"/>
+      <c r="Q318" s="2"/>
+      <c r="R318" s="2"/>
+    </row>
+    <row r="319" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A319" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="B319" s="3" t="s">
+        <v>582</v>
+      </c>
+      <c r="C319" s="3"/>
+      <c r="F319" s="3"/>
+      <c r="G319" s="3"/>
+      <c r="H319" s="3"/>
+      <c r="I319" s="3"/>
+      <c r="J319" s="3"/>
+      <c r="K319" s="3"/>
+      <c r="L319" s="6"/>
+      <c r="M319" s="3"/>
+      <c r="N319" s="6"/>
+      <c r="O319" s="3"/>
+      <c r="P319" s="3"/>
+      <c r="Q319" s="3"/>
+      <c r="R319" s="3"/>
+    </row>
+    <row r="320" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A320" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="B320" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="C320" s="2"/>
+      <c r="F320" s="2"/>
+      <c r="G320" s="2"/>
+      <c r="H320" s="2"/>
+      <c r="I320" s="2"/>
+      <c r="J320" s="2"/>
+      <c r="K320" s="2"/>
+      <c r="L320" s="5"/>
+      <c r="M320" s="2"/>
+      <c r="N320" s="5"/>
+      <c r="O320" s="2"/>
+      <c r="P320" s="2"/>
+      <c r="Q320" s="2"/>
+      <c r="R320" s="2"/>
+    </row>
+    <row r="321" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A321" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="B321" s="3" t="s">
+        <v>586</v>
+      </c>
+      <c r="C321" s="3"/>
+      <c r="F321" s="3"/>
+      <c r="G321" s="3"/>
+      <c r="H321" s="3"/>
+      <c r="I321" s="3"/>
+      <c r="J321" s="3"/>
+      <c r="K321" s="3"/>
+      <c r="L321" s="6"/>
+      <c r="M321" s="3"/>
+      <c r="N321" s="6"/>
+      <c r="O321" s="3"/>
+      <c r="P321" s="3"/>
+      <c r="Q321" s="3"/>
+      <c r="R321" s="3"/>
+    </row>
+    <row r="322" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A322" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="B322" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="C322" s="2"/>
+      <c r="F322" s="2"/>
+      <c r="G322" s="2"/>
+      <c r="H322" s="2"/>
+      <c r="I322" s="2"/>
+      <c r="J322" s="2"/>
+      <c r="K322" s="2"/>
+      <c r="L322" s="5"/>
+      <c r="M322" s="2"/>
+      <c r="N322" s="5"/>
+      <c r="O322" s="2"/>
+      <c r="P322" s="2"/>
+      <c r="Q322" s="2"/>
+      <c r="R322" s="2"/>
+    </row>
+    <row r="323" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A323" s="3" t="s">
+        <v>589</v>
+      </c>
+      <c r="B323" s="3" t="s">
+        <v>590</v>
+      </c>
+      <c r="C323" s="3"/>
+      <c r="F323" s="3"/>
+      <c r="G323" s="3"/>
+      <c r="H323" s="3"/>
+      <c r="I323" s="3"/>
+      <c r="J323" s="3"/>
+      <c r="K323" s="3"/>
+      <c r="L323" s="6"/>
+      <c r="M323" s="3"/>
+      <c r="N323" s="6"/>
+      <c r="O323" s="3"/>
+      <c r="P323" s="3"/>
+      <c r="Q323" s="3"/>
+      <c r="R323" s="3"/>
+    </row>
+    <row r="324" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A324" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="B324" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="C324" s="2"/>
+      <c r="F324" s="2"/>
+      <c r="G324" s="2"/>
+      <c r="H324" s="2"/>
+      <c r="I324" s="2"/>
+      <c r="J324" s="2"/>
+      <c r="K324" s="2"/>
+      <c r="L324" s="5"/>
+      <c r="M324" s="2"/>
+      <c r="N324" s="5"/>
+      <c r="O324" s="2"/>
+      <c r="P324" s="2"/>
+      <c r="Q324" s="2"/>
+      <c r="R324" s="2"/>
+    </row>
+    <row r="325" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A325" s="3" t="s">
+        <v>593</v>
+      </c>
+      <c r="B325" s="3" t="s">
+        <v>594</v>
+      </c>
+      <c r="C325" s="3"/>
+      <c r="F325" s="3"/>
+      <c r="G325" s="3"/>
+      <c r="H325" s="3"/>
+      <c r="I325" s="3"/>
+      <c r="J325" s="3"/>
+      <c r="K325" s="3"/>
+      <c r="L325" s="6"/>
+      <c r="M325" s="3"/>
+      <c r="N325" s="6"/>
+      <c r="O325" s="3"/>
+      <c r="P325" s="3"/>
+      <c r="Q325" s="3"/>
+      <c r="R325" s="3"/>
+    </row>
+    <row r="326" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A326" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B326" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="C326" s="2"/>
+      <c r="F326" s="2"/>
+      <c r="G326" s="2"/>
+      <c r="H326" s="2"/>
+      <c r="I326" s="2"/>
+      <c r="J326" s="2"/>
+      <c r="K326" s="2"/>
+      <c r="L326" s="5"/>
+      <c r="M326" s="2"/>
+      <c r="N326" s="5"/>
+      <c r="O326" s="2"/>
+      <c r="P326" s="2"/>
+      <c r="Q326" s="2"/>
+      <c r="R326" s="2"/>
+    </row>
+    <row r="327" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A327" s="3" t="s">
+        <v>597</v>
+      </c>
+      <c r="B327" s="3" t="s">
+        <v>598</v>
+      </c>
+      <c r="C327" s="3"/>
+      <c r="F327" s="3"/>
+      <c r="G327" s="3"/>
+      <c r="H327" s="3"/>
+      <c r="I327" s="3"/>
+      <c r="J327" s="3"/>
+      <c r="K327" s="3"/>
+      <c r="L327" s="6"/>
+      <c r="M327" s="3"/>
+      <c r="N327" s="6"/>
+      <c r="O327" s="3"/>
+      <c r="P327" s="3"/>
+      <c r="Q327" s="3"/>
+      <c r="R327" s="3"/>
+    </row>
+    <row r="328" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A328" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="B328" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="C328" s="2"/>
+      <c r="F328" s="2"/>
+      <c r="G328" s="2"/>
+      <c r="H328" s="2"/>
+      <c r="I328" s="2"/>
+      <c r="J328" s="2"/>
+      <c r="K328" s="2"/>
+      <c r="L328" s="5"/>
+      <c r="M328" s="2"/>
+      <c r="N328" s="5"/>
+      <c r="O328" s="2"/>
+      <c r="P328" s="2"/>
+      <c r="Q328" s="2"/>
+      <c r="R328" s="2"/>
+    </row>
+    <row r="329" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A329" s="3" t="s">
+        <v>601</v>
+      </c>
+      <c r="B329" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="C329" s="3"/>
+      <c r="F329" s="3"/>
+      <c r="G329" s="3"/>
+      <c r="H329" s="3"/>
+      <c r="I329" s="3"/>
+      <c r="J329" s="3"/>
+      <c r="K329" s="3"/>
+      <c r="L329" s="6"/>
+      <c r="M329" s="3"/>
+      <c r="N329" s="6"/>
+      <c r="O329" s="3"/>
+      <c r="P329" s="3"/>
+      <c r="Q329" s="3"/>
+      <c r="R329" s="3"/>
+    </row>
+    <row r="330" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A330" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="B330" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="C330" s="2"/>
+      <c r="F330" s="2"/>
+      <c r="G330" s="2"/>
+      <c r="H330" s="2"/>
+      <c r="I330" s="2"/>
+      <c r="J330" s="2"/>
+      <c r="K330" s="2"/>
+      <c r="L330" s="5"/>
+      <c r="M330" s="2"/>
+      <c r="N330" s="5"/>
+      <c r="O330" s="2"/>
+      <c r="P330" s="2"/>
+      <c r="Q330" s="2"/>
+      <c r="R330" s="2"/>
+    </row>
+    <row r="331" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B331" s="4"/>
+      <c r="C331" s="3"/>
+      <c r="F331" s="3"/>
+      <c r="G331" s="3"/>
+      <c r="H331" s="3"/>
+      <c r="I331" s="3"/>
+      <c r="J331" s="3"/>
+      <c r="K331" s="3"/>
+      <c r="L331" s="6"/>
+      <c r="M331" s="3"/>
+      <c r="N331" s="6"/>
+      <c r="O331" s="3"/>
+      <c r="P331" s="3"/>
+      <c r="Q331" s="3"/>
+      <c r="R331" s="3"/>
+    </row>
+    <row r="332" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B332" s="4"/>
+      <c r="C332" s="2"/>
+      <c r="F332" s="2"/>
+      <c r="G332" s="2"/>
+      <c r="H332" s="2"/>
+      <c r="I332" s="2"/>
+      <c r="J332" s="2"/>
+      <c r="K332" s="2"/>
+      <c r="L332" s="5"/>
+      <c r="M332" s="2"/>
+      <c r="N332" s="5"/>
+      <c r="O332" s="2"/>
+      <c r="P332" s="2"/>
+      <c r="Q332" s="2"/>
+      <c r="R332" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
add error page in download
</commit_message>
<xml_diff>
--- a/cache/sepidar_food_code.xlsx
+++ b/cache/sepidar_food_code.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\milad\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\milad\Desktop\seketala\cache\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5CBF922-B4E7-436A-B806-78FD705E1D87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57359799-3000-414E-A18F-1C97E5676880}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="620">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="621">
   <si>
     <t>كد</t>
   </si>
@@ -1885,6 +1885,9 @@
   </si>
   <si>
     <t>آب معدني</t>
+  </si>
+  <si>
+    <t>سس سالاد ژامبون و پنير</t>
   </si>
 </sst>
 </file>
@@ -1942,7 +1945,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1950,6 +1953,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="4" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="47" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2230,11 +2234,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R331"/>
+  <dimension ref="A1:AB726"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.140625" customWidth="1"/>
+    <col min="4" max="4" width="31" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -5458,7 +5463,12 @@
       <c r="R329" s="2"/>
     </row>
     <row r="330" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B330" s="4"/>
+      <c r="A330">
+        <v>3000032</v>
+      </c>
+      <c r="B330" s="2" t="s">
+        <v>620</v>
+      </c>
       <c r="C330" s="3"/>
       <c r="F330" s="3"/>
       <c r="G330" s="3"/>
@@ -5491,6 +5501,1554 @@
       <c r="Q331" s="2"/>
       <c r="R331" s="2"/>
     </row>
+    <row r="340" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z340" s="7"/>
+      <c r="AB340" s="7"/>
+    </row>
+    <row r="341" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z341" s="7"/>
+      <c r="AB341" s="7"/>
+    </row>
+    <row r="342" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z342" s="7"/>
+      <c r="AB342" s="7"/>
+    </row>
+    <row r="343" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z343" s="7"/>
+      <c r="AB343" s="7"/>
+    </row>
+    <row r="344" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z344" s="7"/>
+      <c r="AB344" s="7"/>
+    </row>
+    <row r="345" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z345" s="7"/>
+      <c r="AB345" s="7"/>
+    </row>
+    <row r="346" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z346" s="7"/>
+      <c r="AB346" s="7"/>
+    </row>
+    <row r="347" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z347" s="7"/>
+      <c r="AB347" s="7"/>
+    </row>
+    <row r="348" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z348" s="7"/>
+      <c r="AB348" s="7"/>
+    </row>
+    <row r="349" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z349" s="7"/>
+      <c r="AB349" s="7"/>
+    </row>
+    <row r="350" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z350" s="7"/>
+      <c r="AB350" s="7"/>
+    </row>
+    <row r="351" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z351" s="7"/>
+      <c r="AB351" s="7"/>
+    </row>
+    <row r="352" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z352" s="7"/>
+      <c r="AB352" s="7"/>
+    </row>
+    <row r="353" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z353" s="7"/>
+      <c r="AB353" s="7"/>
+    </row>
+    <row r="354" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z354" s="7"/>
+      <c r="AB354" s="7"/>
+    </row>
+    <row r="355" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z355" s="7"/>
+      <c r="AB355" s="7"/>
+    </row>
+    <row r="356" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z356" s="7"/>
+      <c r="AB356" s="7"/>
+    </row>
+    <row r="357" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z357" s="7"/>
+      <c r="AB357" s="7"/>
+    </row>
+    <row r="358" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z358" s="7"/>
+      <c r="AB358" s="7"/>
+    </row>
+    <row r="359" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z359" s="7"/>
+      <c r="AB359" s="7"/>
+    </row>
+    <row r="360" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z360" s="7"/>
+      <c r="AB360" s="7"/>
+    </row>
+    <row r="361" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z361" s="7"/>
+      <c r="AB361" s="7"/>
+    </row>
+    <row r="362" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z362" s="7"/>
+      <c r="AB362" s="7"/>
+    </row>
+    <row r="363" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z363" s="7"/>
+      <c r="AB363" s="7"/>
+    </row>
+    <row r="364" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z364" s="7"/>
+      <c r="AB364" s="7"/>
+    </row>
+    <row r="365" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z365" s="7"/>
+      <c r="AB365" s="7"/>
+    </row>
+    <row r="366" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z366" s="7"/>
+      <c r="AB366" s="7"/>
+    </row>
+    <row r="367" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z367" s="7"/>
+      <c r="AB367" s="7"/>
+    </row>
+    <row r="368" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z368" s="7"/>
+      <c r="AB368" s="7"/>
+    </row>
+    <row r="369" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z369" s="7"/>
+      <c r="AB369" s="7"/>
+    </row>
+    <row r="370" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z370" s="7"/>
+      <c r="AB370" s="7"/>
+    </row>
+    <row r="371" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z371" s="7"/>
+      <c r="AB371" s="7"/>
+    </row>
+    <row r="372" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z372" s="7"/>
+      <c r="AB372" s="7"/>
+    </row>
+    <row r="373" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z373" s="7"/>
+      <c r="AB373" s="7"/>
+    </row>
+    <row r="374" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z374" s="7"/>
+      <c r="AB374" s="7"/>
+    </row>
+    <row r="375" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z375" s="7"/>
+      <c r="AB375" s="7"/>
+    </row>
+    <row r="376" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z376" s="7"/>
+      <c r="AB376" s="7"/>
+    </row>
+    <row r="377" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z377" s="7"/>
+      <c r="AB377" s="7"/>
+    </row>
+    <row r="378" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z378" s="7"/>
+      <c r="AB378" s="7"/>
+    </row>
+    <row r="379" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z379" s="7"/>
+      <c r="AB379" s="7"/>
+    </row>
+    <row r="380" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z380" s="7"/>
+      <c r="AB380" s="7"/>
+    </row>
+    <row r="381" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z381" s="7"/>
+      <c r="AB381" s="7"/>
+    </row>
+    <row r="382" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z382" s="7"/>
+      <c r="AB382" s="7"/>
+    </row>
+    <row r="383" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z383" s="7"/>
+      <c r="AB383" s="7"/>
+    </row>
+    <row r="384" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z384" s="7"/>
+      <c r="AB384" s="7"/>
+    </row>
+    <row r="385" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z385" s="7"/>
+      <c r="AB385" s="7"/>
+    </row>
+    <row r="386" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z386" s="7"/>
+      <c r="AB386" s="7"/>
+    </row>
+    <row r="387" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z387" s="7"/>
+      <c r="AB387" s="7"/>
+    </row>
+    <row r="388" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z388" s="7"/>
+      <c r="AB388" s="7"/>
+    </row>
+    <row r="389" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z389" s="7"/>
+      <c r="AB389" s="7"/>
+    </row>
+    <row r="390" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z390" s="7"/>
+      <c r="AB390" s="7"/>
+    </row>
+    <row r="391" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z391" s="7"/>
+      <c r="AB391" s="7"/>
+    </row>
+    <row r="392" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z392" s="7"/>
+      <c r="AB392" s="7"/>
+    </row>
+    <row r="393" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z393" s="7"/>
+      <c r="AB393" s="7"/>
+    </row>
+    <row r="394" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z394" s="7"/>
+      <c r="AB394" s="7"/>
+    </row>
+    <row r="395" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z395" s="7"/>
+      <c r="AB395" s="7"/>
+    </row>
+    <row r="396" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z396" s="7"/>
+      <c r="AB396" s="7"/>
+    </row>
+    <row r="397" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z397" s="7"/>
+      <c r="AB397" s="7"/>
+    </row>
+    <row r="398" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z398" s="7"/>
+      <c r="AB398" s="7"/>
+    </row>
+    <row r="399" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z399" s="7"/>
+      <c r="AB399" s="7"/>
+    </row>
+    <row r="400" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z400" s="7"/>
+      <c r="AB400" s="7"/>
+    </row>
+    <row r="401" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z401" s="7"/>
+      <c r="AB401" s="7"/>
+    </row>
+    <row r="402" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z402" s="7"/>
+      <c r="AB402" s="7"/>
+    </row>
+    <row r="403" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z403" s="7"/>
+      <c r="AB403" s="7"/>
+    </row>
+    <row r="404" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z404" s="7"/>
+      <c r="AB404" s="7"/>
+    </row>
+    <row r="405" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z405" s="7"/>
+      <c r="AB405" s="7"/>
+    </row>
+    <row r="406" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z406" s="7"/>
+      <c r="AB406" s="7"/>
+    </row>
+    <row r="407" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z407" s="7"/>
+      <c r="AB407" s="7"/>
+    </row>
+    <row r="408" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z408" s="7"/>
+      <c r="AB408" s="7"/>
+    </row>
+    <row r="409" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z409" s="7"/>
+      <c r="AB409" s="7"/>
+    </row>
+    <row r="410" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z410" s="7"/>
+      <c r="AB410" s="7"/>
+    </row>
+    <row r="411" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z411" s="7"/>
+      <c r="AB411" s="7"/>
+    </row>
+    <row r="412" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z412" s="7"/>
+      <c r="AB412" s="7"/>
+    </row>
+    <row r="413" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z413" s="7"/>
+      <c r="AB413" s="7"/>
+    </row>
+    <row r="414" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z414" s="7"/>
+      <c r="AB414" s="7"/>
+    </row>
+    <row r="415" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z415" s="7"/>
+      <c r="AB415" s="7"/>
+    </row>
+    <row r="416" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z416" s="7"/>
+      <c r="AB416" s="7"/>
+    </row>
+    <row r="417" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z417" s="7"/>
+      <c r="AB417" s="7"/>
+    </row>
+    <row r="418" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z418" s="7"/>
+      <c r="AB418" s="7"/>
+    </row>
+    <row r="419" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z419" s="7"/>
+      <c r="AB419" s="7"/>
+    </row>
+    <row r="420" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z420" s="7"/>
+      <c r="AB420" s="7"/>
+    </row>
+    <row r="421" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z421" s="7"/>
+      <c r="AB421" s="7"/>
+    </row>
+    <row r="422" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z422" s="7"/>
+      <c r="AB422" s="7"/>
+    </row>
+    <row r="423" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z423" s="7"/>
+      <c r="AB423" s="7"/>
+    </row>
+    <row r="424" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z424" s="7"/>
+      <c r="AB424" s="7"/>
+    </row>
+    <row r="425" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z425" s="7"/>
+      <c r="AB425" s="7"/>
+    </row>
+    <row r="426" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z426" s="7"/>
+      <c r="AB426" s="7"/>
+    </row>
+    <row r="427" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z427" s="7"/>
+      <c r="AB427" s="7"/>
+    </row>
+    <row r="428" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z428" s="7"/>
+      <c r="AB428" s="7"/>
+    </row>
+    <row r="429" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z429" s="7"/>
+      <c r="AB429" s="7"/>
+    </row>
+    <row r="430" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z430" s="7"/>
+      <c r="AB430" s="7"/>
+    </row>
+    <row r="431" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z431" s="7"/>
+      <c r="AB431" s="7"/>
+    </row>
+    <row r="432" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z432" s="7"/>
+      <c r="AB432" s="7"/>
+    </row>
+    <row r="433" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z433" s="7"/>
+      <c r="AB433" s="7"/>
+    </row>
+    <row r="434" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z434" s="7"/>
+      <c r="AB434" s="7"/>
+    </row>
+    <row r="435" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z435" s="7"/>
+      <c r="AB435" s="7"/>
+    </row>
+    <row r="436" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z436" s="7"/>
+      <c r="AB436" s="7"/>
+    </row>
+    <row r="437" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z437" s="7"/>
+      <c r="AB437" s="7"/>
+    </row>
+    <row r="438" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z438" s="7"/>
+      <c r="AB438" s="7"/>
+    </row>
+    <row r="439" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z439" s="7"/>
+      <c r="AB439" s="7"/>
+    </row>
+    <row r="440" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z440" s="7"/>
+      <c r="AB440" s="7"/>
+    </row>
+    <row r="441" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z441" s="7"/>
+      <c r="AB441" s="7"/>
+    </row>
+    <row r="442" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z442" s="7"/>
+      <c r="AB442" s="7"/>
+    </row>
+    <row r="443" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z443" s="7"/>
+      <c r="AB443" s="7"/>
+    </row>
+    <row r="444" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z444" s="7"/>
+      <c r="AB444" s="7"/>
+    </row>
+    <row r="445" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z445" s="7"/>
+      <c r="AB445" s="7"/>
+    </row>
+    <row r="446" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z446" s="7"/>
+      <c r="AB446" s="7"/>
+    </row>
+    <row r="447" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z447" s="7"/>
+      <c r="AB447" s="7"/>
+    </row>
+    <row r="448" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z448" s="7"/>
+      <c r="AB448" s="7"/>
+    </row>
+    <row r="449" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z449" s="7"/>
+      <c r="AB449" s="7"/>
+    </row>
+    <row r="450" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z450" s="7"/>
+      <c r="AB450" s="7"/>
+    </row>
+    <row r="451" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z451" s="7"/>
+      <c r="AB451" s="7"/>
+    </row>
+    <row r="452" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z452" s="7"/>
+      <c r="AB452" s="7"/>
+    </row>
+    <row r="453" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z453" s="7"/>
+      <c r="AB453" s="7"/>
+    </row>
+    <row r="454" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z454" s="7"/>
+      <c r="AB454" s="7"/>
+    </row>
+    <row r="455" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z455" s="7"/>
+      <c r="AB455" s="7"/>
+    </row>
+    <row r="456" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z456" s="7"/>
+      <c r="AB456" s="7"/>
+    </row>
+    <row r="457" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z457" s="7"/>
+      <c r="AB457" s="7"/>
+    </row>
+    <row r="458" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z458" s="7"/>
+      <c r="AB458" s="7"/>
+    </row>
+    <row r="459" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z459" s="7"/>
+      <c r="AB459" s="7"/>
+    </row>
+    <row r="460" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z460" s="7"/>
+      <c r="AB460" s="7"/>
+    </row>
+    <row r="461" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z461" s="7"/>
+      <c r="AB461" s="7"/>
+    </row>
+    <row r="462" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z462" s="7"/>
+      <c r="AB462" s="7"/>
+    </row>
+    <row r="463" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z463" s="7"/>
+      <c r="AB463" s="7"/>
+    </row>
+    <row r="464" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z464" s="7"/>
+      <c r="AB464" s="7"/>
+    </row>
+    <row r="465" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z465" s="7"/>
+      <c r="AB465" s="7"/>
+    </row>
+    <row r="466" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z466" s="7"/>
+      <c r="AB466" s="7"/>
+    </row>
+    <row r="467" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z467" s="7"/>
+      <c r="AB467" s="7"/>
+    </row>
+    <row r="468" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z468" s="7"/>
+      <c r="AB468" s="7"/>
+    </row>
+    <row r="469" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z469" s="7"/>
+      <c r="AB469" s="7"/>
+    </row>
+    <row r="470" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z470" s="7"/>
+      <c r="AB470" s="7"/>
+    </row>
+    <row r="471" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z471" s="7"/>
+      <c r="AB471" s="7"/>
+    </row>
+    <row r="472" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z472" s="7"/>
+      <c r="AB472" s="7"/>
+    </row>
+    <row r="473" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z473" s="7"/>
+      <c r="AB473" s="7"/>
+    </row>
+    <row r="474" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z474" s="7"/>
+      <c r="AB474" s="7"/>
+    </row>
+    <row r="475" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z475" s="7"/>
+      <c r="AB475" s="7"/>
+    </row>
+    <row r="476" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z476" s="7"/>
+      <c r="AB476" s="7"/>
+    </row>
+    <row r="477" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z477" s="7"/>
+      <c r="AB477" s="7"/>
+    </row>
+    <row r="478" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z478" s="7"/>
+      <c r="AB478" s="7"/>
+    </row>
+    <row r="479" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z479" s="7"/>
+      <c r="AB479" s="7"/>
+    </row>
+    <row r="480" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z480" s="7"/>
+      <c r="AB480" s="7"/>
+    </row>
+    <row r="481" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z481" s="7"/>
+      <c r="AB481" s="7"/>
+    </row>
+    <row r="482" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z482" s="7"/>
+      <c r="AB482" s="7"/>
+    </row>
+    <row r="483" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z483" s="7"/>
+      <c r="AB483" s="7"/>
+    </row>
+    <row r="484" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z484" s="7"/>
+      <c r="AB484" s="7"/>
+    </row>
+    <row r="485" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z485" s="7"/>
+      <c r="AB485" s="7"/>
+    </row>
+    <row r="486" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z486" s="7"/>
+      <c r="AB486" s="7"/>
+    </row>
+    <row r="487" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z487" s="7"/>
+      <c r="AB487" s="7"/>
+    </row>
+    <row r="488" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z488" s="7"/>
+      <c r="AB488" s="7"/>
+    </row>
+    <row r="489" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z489" s="7"/>
+      <c r="AB489" s="7"/>
+    </row>
+    <row r="490" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z490" s="7"/>
+      <c r="AB490" s="7"/>
+    </row>
+    <row r="491" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z491" s="7"/>
+      <c r="AB491" s="7"/>
+    </row>
+    <row r="492" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z492" s="7"/>
+      <c r="AB492" s="7"/>
+    </row>
+    <row r="493" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z493" s="7"/>
+      <c r="AB493" s="7"/>
+    </row>
+    <row r="494" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z494" s="7"/>
+      <c r="AB494" s="7"/>
+    </row>
+    <row r="495" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z495" s="7"/>
+      <c r="AB495" s="7"/>
+    </row>
+    <row r="496" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z496" s="7"/>
+      <c r="AB496" s="7"/>
+    </row>
+    <row r="497" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z497" s="7"/>
+      <c r="AB497" s="7"/>
+    </row>
+    <row r="498" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z498" s="7"/>
+      <c r="AB498" s="7"/>
+    </row>
+    <row r="499" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z499" s="7"/>
+      <c r="AB499" s="7"/>
+    </row>
+    <row r="500" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z500" s="7"/>
+      <c r="AB500" s="7"/>
+    </row>
+    <row r="501" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z501" s="7"/>
+      <c r="AB501" s="7"/>
+    </row>
+    <row r="502" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z502" s="7"/>
+      <c r="AB502" s="7"/>
+    </row>
+    <row r="503" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z503" s="7"/>
+      <c r="AB503" s="7"/>
+    </row>
+    <row r="504" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z504" s="7"/>
+      <c r="AB504" s="7"/>
+    </row>
+    <row r="505" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z505" s="7"/>
+      <c r="AB505" s="7"/>
+    </row>
+    <row r="506" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z506" s="7"/>
+      <c r="AB506" s="7"/>
+    </row>
+    <row r="507" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z507" s="7"/>
+      <c r="AB507" s="7"/>
+    </row>
+    <row r="508" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z508" s="7"/>
+      <c r="AB508" s="7"/>
+    </row>
+    <row r="509" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z509" s="7"/>
+      <c r="AB509" s="7"/>
+    </row>
+    <row r="510" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z510" s="7"/>
+      <c r="AB510" s="7"/>
+    </row>
+    <row r="511" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z511" s="7"/>
+      <c r="AB511" s="7"/>
+    </row>
+    <row r="512" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z512" s="7"/>
+      <c r="AB512" s="7"/>
+    </row>
+    <row r="513" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z513" s="7"/>
+      <c r="AB513" s="7"/>
+    </row>
+    <row r="514" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z514" s="7"/>
+      <c r="AB514" s="7"/>
+    </row>
+    <row r="515" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z515" s="7"/>
+      <c r="AB515" s="7"/>
+    </row>
+    <row r="516" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z516" s="7"/>
+      <c r="AB516" s="7"/>
+    </row>
+    <row r="517" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z517" s="7"/>
+      <c r="AB517" s="7"/>
+    </row>
+    <row r="518" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z518" s="7"/>
+      <c r="AB518" s="7"/>
+    </row>
+    <row r="519" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z519" s="7"/>
+      <c r="AB519" s="7"/>
+    </row>
+    <row r="520" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z520" s="7"/>
+      <c r="AB520" s="7"/>
+    </row>
+    <row r="521" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z521" s="7"/>
+      <c r="AB521" s="7"/>
+    </row>
+    <row r="522" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z522" s="7"/>
+      <c r="AB522" s="7"/>
+    </row>
+    <row r="523" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z523" s="7"/>
+      <c r="AB523" s="7"/>
+    </row>
+    <row r="524" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z524" s="7"/>
+      <c r="AB524" s="7"/>
+    </row>
+    <row r="525" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z525" s="7"/>
+      <c r="AB525" s="7"/>
+    </row>
+    <row r="526" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z526" s="7"/>
+      <c r="AB526" s="7"/>
+    </row>
+    <row r="527" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z527" s="7"/>
+      <c r="AB527" s="7"/>
+    </row>
+    <row r="528" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z528" s="7"/>
+      <c r="AB528" s="7"/>
+    </row>
+    <row r="529" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z529" s="7"/>
+      <c r="AB529" s="7"/>
+    </row>
+    <row r="530" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z530" s="7"/>
+      <c r="AB530" s="7"/>
+    </row>
+    <row r="531" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z531" s="7"/>
+      <c r="AB531" s="7"/>
+    </row>
+    <row r="532" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z532" s="7"/>
+      <c r="AB532" s="7"/>
+    </row>
+    <row r="533" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z533" s="7"/>
+      <c r="AB533" s="7"/>
+    </row>
+    <row r="534" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z534" s="7"/>
+      <c r="AB534" s="7"/>
+    </row>
+    <row r="535" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z535" s="7"/>
+      <c r="AB535" s="7"/>
+    </row>
+    <row r="536" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z536" s="7"/>
+      <c r="AB536" s="7"/>
+    </row>
+    <row r="537" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z537" s="7"/>
+      <c r="AB537" s="7"/>
+    </row>
+    <row r="538" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z538" s="7"/>
+      <c r="AB538" s="7"/>
+    </row>
+    <row r="539" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z539" s="7"/>
+      <c r="AB539" s="7"/>
+    </row>
+    <row r="540" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z540" s="7"/>
+      <c r="AB540" s="7"/>
+    </row>
+    <row r="541" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z541" s="7"/>
+      <c r="AB541" s="7"/>
+    </row>
+    <row r="542" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z542" s="7"/>
+      <c r="AB542" s="7"/>
+    </row>
+    <row r="543" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z543" s="7"/>
+      <c r="AB543" s="7"/>
+    </row>
+    <row r="544" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z544" s="7"/>
+      <c r="AB544" s="7"/>
+    </row>
+    <row r="545" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z545" s="7"/>
+      <c r="AB545" s="7"/>
+    </row>
+    <row r="546" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z546" s="7"/>
+      <c r="AB546" s="7"/>
+    </row>
+    <row r="547" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z547" s="7"/>
+      <c r="AB547" s="7"/>
+    </row>
+    <row r="548" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z548" s="7"/>
+      <c r="AB548" s="7"/>
+    </row>
+    <row r="549" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z549" s="7"/>
+      <c r="AB549" s="7"/>
+    </row>
+    <row r="550" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z550" s="7"/>
+      <c r="AB550" s="7"/>
+    </row>
+    <row r="551" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z551" s="7"/>
+      <c r="AB551" s="7"/>
+    </row>
+    <row r="552" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z552" s="7"/>
+      <c r="AB552" s="7"/>
+    </row>
+    <row r="553" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z553" s="7"/>
+      <c r="AB553" s="7"/>
+    </row>
+    <row r="554" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z554" s="7"/>
+      <c r="AB554" s="7"/>
+    </row>
+    <row r="555" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z555" s="7"/>
+      <c r="AB555" s="7"/>
+    </row>
+    <row r="556" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z556" s="7"/>
+      <c r="AB556" s="7"/>
+    </row>
+    <row r="557" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z557" s="7"/>
+      <c r="AB557" s="7"/>
+    </row>
+    <row r="558" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z558" s="7"/>
+      <c r="AB558" s="7"/>
+    </row>
+    <row r="559" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z559" s="7"/>
+      <c r="AB559" s="7"/>
+    </row>
+    <row r="560" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z560" s="7"/>
+      <c r="AB560" s="7"/>
+    </row>
+    <row r="561" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z561" s="7"/>
+      <c r="AB561" s="7"/>
+    </row>
+    <row r="562" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z562" s="7"/>
+      <c r="AB562" s="7"/>
+    </row>
+    <row r="563" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z563" s="7"/>
+      <c r="AB563" s="7"/>
+    </row>
+    <row r="564" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z564" s="7"/>
+      <c r="AB564" s="7"/>
+    </row>
+    <row r="565" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z565" s="7"/>
+      <c r="AB565" s="7"/>
+    </row>
+    <row r="566" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z566" s="7"/>
+      <c r="AB566" s="7"/>
+    </row>
+    <row r="567" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z567" s="7"/>
+      <c r="AB567" s="7"/>
+    </row>
+    <row r="568" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z568" s="7"/>
+      <c r="AB568" s="7"/>
+    </row>
+    <row r="569" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z569" s="7"/>
+      <c r="AB569" s="7"/>
+    </row>
+    <row r="570" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z570" s="7"/>
+      <c r="AB570" s="7"/>
+    </row>
+    <row r="571" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z571" s="7"/>
+      <c r="AB571" s="7"/>
+    </row>
+    <row r="572" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z572" s="7"/>
+      <c r="AB572" s="7"/>
+    </row>
+    <row r="573" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z573" s="7"/>
+      <c r="AB573" s="7"/>
+    </row>
+    <row r="574" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z574" s="7"/>
+      <c r="AB574" s="7"/>
+    </row>
+    <row r="575" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z575" s="7"/>
+      <c r="AB575" s="7"/>
+    </row>
+    <row r="576" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z576" s="7"/>
+      <c r="AB576" s="7"/>
+    </row>
+    <row r="577" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z577" s="7"/>
+      <c r="AB577" s="7"/>
+    </row>
+    <row r="578" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z578" s="7"/>
+      <c r="AB578" s="7"/>
+    </row>
+    <row r="579" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z579" s="7"/>
+      <c r="AB579" s="7"/>
+    </row>
+    <row r="580" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z580" s="7"/>
+      <c r="AB580" s="7"/>
+    </row>
+    <row r="581" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z581" s="7"/>
+      <c r="AB581" s="7"/>
+    </row>
+    <row r="582" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z582" s="7"/>
+      <c r="AB582" s="7"/>
+    </row>
+    <row r="583" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z583" s="7"/>
+      <c r="AB583" s="7"/>
+    </row>
+    <row r="584" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z584" s="7"/>
+      <c r="AB584" s="7"/>
+    </row>
+    <row r="585" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z585" s="7"/>
+      <c r="AB585" s="7"/>
+    </row>
+    <row r="586" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z586" s="7"/>
+      <c r="AB586" s="7"/>
+    </row>
+    <row r="587" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z587" s="7"/>
+      <c r="AB587" s="7"/>
+    </row>
+    <row r="588" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z588" s="7"/>
+      <c r="AB588" s="7"/>
+    </row>
+    <row r="589" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z589" s="7"/>
+      <c r="AB589" s="7"/>
+    </row>
+    <row r="590" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z590" s="7"/>
+      <c r="AB590" s="7"/>
+    </row>
+    <row r="591" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z591" s="7"/>
+      <c r="AB591" s="7"/>
+    </row>
+    <row r="592" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z592" s="7"/>
+      <c r="AB592" s="7"/>
+    </row>
+    <row r="593" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z593" s="7"/>
+      <c r="AB593" s="7"/>
+    </row>
+    <row r="594" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z594" s="7"/>
+      <c r="AB594" s="7"/>
+    </row>
+    <row r="595" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z595" s="7"/>
+      <c r="AB595" s="7"/>
+    </row>
+    <row r="596" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z596" s="7"/>
+      <c r="AB596" s="7"/>
+    </row>
+    <row r="597" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z597" s="7"/>
+      <c r="AB597" s="7"/>
+    </row>
+    <row r="598" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z598" s="7"/>
+      <c r="AB598" s="7"/>
+    </row>
+    <row r="599" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z599" s="7"/>
+      <c r="AB599" s="7"/>
+    </row>
+    <row r="600" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z600" s="7"/>
+      <c r="AB600" s="7"/>
+    </row>
+    <row r="601" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z601" s="7"/>
+      <c r="AB601" s="7"/>
+    </row>
+    <row r="602" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z602" s="7"/>
+      <c r="AB602" s="7"/>
+    </row>
+    <row r="603" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z603" s="7"/>
+      <c r="AB603" s="7"/>
+    </row>
+    <row r="604" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z604" s="7"/>
+      <c r="AB604" s="7"/>
+    </row>
+    <row r="605" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z605" s="7"/>
+      <c r="AB605" s="7"/>
+    </row>
+    <row r="606" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z606" s="7"/>
+      <c r="AB606" s="7"/>
+    </row>
+    <row r="607" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z607" s="7"/>
+      <c r="AB607" s="7"/>
+    </row>
+    <row r="608" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z608" s="7"/>
+      <c r="AB608" s="7"/>
+    </row>
+    <row r="609" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z609" s="7"/>
+      <c r="AB609" s="7"/>
+    </row>
+    <row r="610" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z610" s="7"/>
+      <c r="AB610" s="7"/>
+    </row>
+    <row r="611" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z611" s="7"/>
+      <c r="AB611" s="7"/>
+    </row>
+    <row r="612" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z612" s="7"/>
+      <c r="AB612" s="7"/>
+    </row>
+    <row r="613" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z613" s="7"/>
+      <c r="AB613" s="7"/>
+    </row>
+    <row r="614" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z614" s="7"/>
+      <c r="AB614" s="7"/>
+    </row>
+    <row r="615" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z615" s="7"/>
+      <c r="AB615" s="7"/>
+    </row>
+    <row r="616" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z616" s="7"/>
+      <c r="AB616" s="7"/>
+    </row>
+    <row r="617" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z617" s="7"/>
+      <c r="AB617" s="7"/>
+    </row>
+    <row r="618" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z618" s="7"/>
+      <c r="AB618" s="7"/>
+    </row>
+    <row r="619" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z619" s="7"/>
+      <c r="AB619" s="7"/>
+    </row>
+    <row r="620" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z620" s="7"/>
+      <c r="AB620" s="7"/>
+    </row>
+    <row r="621" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z621" s="7"/>
+      <c r="AB621" s="7"/>
+    </row>
+    <row r="622" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z622" s="7"/>
+      <c r="AB622" s="7"/>
+    </row>
+    <row r="623" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z623" s="7"/>
+      <c r="AB623" s="7"/>
+    </row>
+    <row r="624" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z624" s="7"/>
+      <c r="AB624" s="7"/>
+    </row>
+    <row r="625" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z625" s="7"/>
+      <c r="AB625" s="7"/>
+    </row>
+    <row r="626" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z626" s="7"/>
+      <c r="AB626" s="7"/>
+    </row>
+    <row r="627" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z627" s="7"/>
+      <c r="AB627" s="7"/>
+    </row>
+    <row r="628" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z628" s="7"/>
+      <c r="AB628" s="7"/>
+    </row>
+    <row r="629" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z629" s="7"/>
+      <c r="AB629" s="7"/>
+    </row>
+    <row r="630" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z630" s="7"/>
+      <c r="AB630" s="7"/>
+    </row>
+    <row r="631" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z631" s="7"/>
+      <c r="AB631" s="7"/>
+    </row>
+    <row r="632" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z632" s="7"/>
+      <c r="AB632" s="7"/>
+    </row>
+    <row r="633" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z633" s="7"/>
+      <c r="AB633" s="7"/>
+    </row>
+    <row r="634" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z634" s="7"/>
+      <c r="AB634" s="7"/>
+    </row>
+    <row r="635" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z635" s="7"/>
+      <c r="AB635" s="7"/>
+    </row>
+    <row r="636" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z636" s="7"/>
+      <c r="AB636" s="7"/>
+    </row>
+    <row r="637" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z637" s="7"/>
+      <c r="AB637" s="7"/>
+    </row>
+    <row r="638" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z638" s="7"/>
+      <c r="AB638" s="7"/>
+    </row>
+    <row r="639" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z639" s="7"/>
+      <c r="AB639" s="7"/>
+    </row>
+    <row r="640" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z640" s="7"/>
+      <c r="AB640" s="7"/>
+    </row>
+    <row r="641" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z641" s="7"/>
+      <c r="AB641" s="7"/>
+    </row>
+    <row r="642" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z642" s="7"/>
+      <c r="AB642" s="7"/>
+    </row>
+    <row r="643" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z643" s="7"/>
+      <c r="AB643" s="7"/>
+    </row>
+    <row r="644" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z644" s="7"/>
+      <c r="AB644" s="7"/>
+    </row>
+    <row r="645" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z645" s="7"/>
+      <c r="AB645" s="7"/>
+    </row>
+    <row r="646" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z646" s="7"/>
+      <c r="AB646" s="7"/>
+    </row>
+    <row r="647" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z647" s="7"/>
+      <c r="AB647" s="7"/>
+    </row>
+    <row r="648" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z648" s="7"/>
+      <c r="AB648" s="7"/>
+    </row>
+    <row r="649" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z649" s="7"/>
+      <c r="AB649" s="7"/>
+    </row>
+    <row r="650" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z650" s="7"/>
+      <c r="AB650" s="7"/>
+    </row>
+    <row r="651" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z651" s="7"/>
+      <c r="AB651" s="7"/>
+    </row>
+    <row r="652" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z652" s="7"/>
+      <c r="AB652" s="7"/>
+    </row>
+    <row r="653" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z653" s="7"/>
+      <c r="AB653" s="7"/>
+    </row>
+    <row r="654" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z654" s="7"/>
+      <c r="AB654" s="7"/>
+    </row>
+    <row r="655" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z655" s="7"/>
+      <c r="AB655" s="7"/>
+    </row>
+    <row r="656" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z656" s="7"/>
+      <c r="AB656" s="7"/>
+    </row>
+    <row r="657" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z657" s="7"/>
+      <c r="AB657" s="7"/>
+    </row>
+    <row r="658" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z658" s="7"/>
+      <c r="AB658" s="7"/>
+    </row>
+    <row r="659" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z659" s="7"/>
+      <c r="AB659" s="7"/>
+    </row>
+    <row r="660" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z660" s="7"/>
+      <c r="AB660" s="7"/>
+    </row>
+    <row r="661" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z661" s="7"/>
+      <c r="AB661" s="7"/>
+    </row>
+    <row r="662" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z662" s="7"/>
+      <c r="AB662" s="7"/>
+    </row>
+    <row r="663" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z663" s="7"/>
+      <c r="AB663" s="7"/>
+    </row>
+    <row r="664" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z664" s="7"/>
+      <c r="AB664" s="7"/>
+    </row>
+    <row r="665" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z665" s="7"/>
+      <c r="AB665" s="7"/>
+    </row>
+    <row r="666" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z666" s="7"/>
+      <c r="AB666" s="7"/>
+    </row>
+    <row r="667" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z667" s="7"/>
+      <c r="AB667" s="7"/>
+    </row>
+    <row r="668" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z668" s="7"/>
+      <c r="AB668" s="7"/>
+    </row>
+    <row r="669" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z669" s="7"/>
+      <c r="AB669" s="7"/>
+    </row>
+    <row r="670" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z670" s="7"/>
+      <c r="AB670" s="7"/>
+    </row>
+    <row r="671" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z671" s="7"/>
+      <c r="AB671" s="7"/>
+    </row>
+    <row r="672" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z672" s="7"/>
+      <c r="AB672" s="7"/>
+    </row>
+    <row r="673" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z673" s="7"/>
+      <c r="AB673" s="7"/>
+    </row>
+    <row r="674" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z674" s="7"/>
+      <c r="AB674" s="7"/>
+    </row>
+    <row r="675" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z675" s="7"/>
+      <c r="AB675" s="7"/>
+    </row>
+    <row r="676" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z676" s="7"/>
+      <c r="AB676" s="7"/>
+    </row>
+    <row r="677" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z677" s="7"/>
+      <c r="AB677" s="7"/>
+    </row>
+    <row r="678" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z678" s="7"/>
+      <c r="AB678" s="7"/>
+    </row>
+    <row r="679" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z679" s="7"/>
+      <c r="AB679" s="7"/>
+    </row>
+    <row r="680" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z680" s="7"/>
+      <c r="AB680" s="7"/>
+    </row>
+    <row r="681" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z681" s="7"/>
+      <c r="AB681" s="7"/>
+    </row>
+    <row r="682" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z682" s="7"/>
+      <c r="AB682" s="7"/>
+    </row>
+    <row r="683" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z683" s="7"/>
+      <c r="AB683" s="7"/>
+    </row>
+    <row r="684" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z684" s="7"/>
+      <c r="AB684" s="7"/>
+    </row>
+    <row r="685" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z685" s="7"/>
+      <c r="AB685" s="7"/>
+    </row>
+    <row r="686" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z686" s="7"/>
+      <c r="AB686" s="7"/>
+    </row>
+    <row r="687" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z687" s="7"/>
+      <c r="AB687" s="7"/>
+    </row>
+    <row r="688" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z688" s="7"/>
+      <c r="AB688" s="7"/>
+    </row>
+    <row r="689" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z689" s="7"/>
+      <c r="AB689" s="7"/>
+    </row>
+    <row r="690" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z690" s="7"/>
+      <c r="AB690" s="7"/>
+    </row>
+    <row r="691" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z691" s="7"/>
+      <c r="AB691" s="7"/>
+    </row>
+    <row r="692" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z692" s="7"/>
+      <c r="AB692" s="7"/>
+    </row>
+    <row r="693" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z693" s="7"/>
+      <c r="AB693" s="7"/>
+    </row>
+    <row r="694" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z694" s="7"/>
+      <c r="AB694" s="7"/>
+    </row>
+    <row r="695" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z695" s="7"/>
+      <c r="AB695" s="7"/>
+    </row>
+    <row r="696" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z696" s="7"/>
+      <c r="AB696" s="7"/>
+    </row>
+    <row r="697" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z697" s="7"/>
+      <c r="AB697" s="7"/>
+    </row>
+    <row r="698" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z698" s="7"/>
+      <c r="AB698" s="7"/>
+    </row>
+    <row r="699" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z699" s="7"/>
+      <c r="AB699" s="7"/>
+    </row>
+    <row r="700" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z700" s="7"/>
+      <c r="AB700" s="7"/>
+    </row>
+    <row r="701" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z701" s="7"/>
+      <c r="AB701" s="7"/>
+    </row>
+    <row r="702" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z702" s="7"/>
+      <c r="AB702" s="7"/>
+    </row>
+    <row r="703" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z703" s="7"/>
+      <c r="AB703" s="7"/>
+    </row>
+    <row r="704" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z704" s="7"/>
+      <c r="AB704" s="7"/>
+    </row>
+    <row r="705" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z705" s="7"/>
+      <c r="AB705" s="7"/>
+    </row>
+    <row r="706" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z706" s="7"/>
+      <c r="AB706" s="7"/>
+    </row>
+    <row r="707" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z707" s="7"/>
+      <c r="AB707" s="7"/>
+    </row>
+    <row r="708" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z708" s="7"/>
+      <c r="AB708" s="7"/>
+    </row>
+    <row r="709" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z709" s="7"/>
+      <c r="AB709" s="7"/>
+    </row>
+    <row r="710" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z710" s="7"/>
+      <c r="AB710" s="7"/>
+    </row>
+    <row r="711" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z711" s="7"/>
+      <c r="AB711" s="7"/>
+    </row>
+    <row r="712" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z712" s="7"/>
+      <c r="AB712" s="7"/>
+    </row>
+    <row r="713" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z713" s="7"/>
+      <c r="AB713" s="7"/>
+    </row>
+    <row r="714" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z714" s="7"/>
+      <c r="AB714" s="7"/>
+    </row>
+    <row r="715" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z715" s="7"/>
+      <c r="AB715" s="7"/>
+    </row>
+    <row r="716" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z716" s="7"/>
+      <c r="AB716" s="7"/>
+    </row>
+    <row r="717" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z717" s="7"/>
+      <c r="AB717" s="7"/>
+    </row>
+    <row r="718" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z718" s="7"/>
+      <c r="AB718" s="7"/>
+    </row>
+    <row r="719" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z719" s="7"/>
+      <c r="AB719" s="7"/>
+    </row>
+    <row r="720" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z720" s="7"/>
+      <c r="AB720" s="7"/>
+    </row>
+    <row r="721" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z721" s="7"/>
+      <c r="AB721" s="7"/>
+    </row>
+    <row r="722" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z722" s="7"/>
+      <c r="AB722" s="7"/>
+    </row>
+    <row r="723" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z723" s="7"/>
+      <c r="AB723" s="7"/>
+    </row>
+    <row r="724" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z724" s="7"/>
+      <c r="AB724" s="7"/>
+    </row>
+    <row r="725" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z725" s="7"/>
+      <c r="AB725" s="7"/>
+    </row>
+    <row r="726" spans="26:28" x14ac:dyDescent="0.25">
+      <c r="Z726" s="7"/>
+      <c r="AB726" s="7"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>